<commit_message>
fix(build): sua signature UpdateAsync trong DoiTacService ve Task<bool> va sua XML comment SecretProtector
</commit_message>
<xml_diff>
--- a/docs/Mau_Bao_Cao_Va_Data_Mapping_QLDA.xlsx
+++ b/docs/Mau_Bao_Cao_Va_Data_Mapping_QLDA.xlsx
@@ -88,6 +88,12 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="00047857"/>
       <sz val="9"/>
     </font>
@@ -95,12 +101,6 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00B45309"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00B91C1C"/>
       <sz val="9"/>
     </font>
     <font>
@@ -140,7 +140,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -167,20 +167,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
-        <bgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF9C3"/>
-        <bgColor rgb="00FEF9C3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-        <bgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00E2E8F0"/>
+        <bgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -245,8 +233,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
-        <bgColor rgb="00E2E8F0"/>
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+        <bgColor rgb="00FEF9C3"/>
       </patternFill>
     </fill>
   </fills>
@@ -276,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -320,18 +314,26 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -340,9 +342,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -357,15 +356,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -377,8 +375,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -758,12 +755,12 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -776,7 +773,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TỔNG HỢP BIỂU MẪU BÁO CÁO THỰC TẾ &amp; MÔ TẢ DATA MAPPING NGUỒN CSDL</t>
+          <t>TỔNG HỢP BIỂU MẪU BÁO CÁO THỰC TẾ &amp; MÔ TẢ DATA MAPPING NGUỒN CSDL (CẬP NHẬT THEO HỆ THỐNG ĐANG CHẠY)</t>
         </is>
       </c>
     </row>
@@ -791,7 +788,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>DANH SÁCH BIỂU MẪU BÁO CÁO &amp; MÔ TẢ ĐÃ CẬP NHẬT THEO THỰC TẾ DỰ ÁN</t>
+          <t>DANH SÁCH BIỂU MẪU BÁO CÁO &amp; MÔ TẢ ĐÃ ĐỒNG BỘ THEO THỰC TẾ PHẦN MỀM</t>
         </is>
       </c>
     </row>
@@ -823,7 +820,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Trạng Thái Cập Nhật</t>
+          <t>Trạng Thái Thực Tế Phần Mềm</t>
         </is>
       </c>
     </row>
@@ -833,12 +830,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Báo cáo 1 - Tiến độ dự án</t>
+          <t>Báo cáo 1: Tiến độ Dự án triển khai</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Theo dõi tiến độ triển khai, thời gian bắt đầu/kết thúc, số ngày còn lại và cảnh báo rủi ro (RAG) theo thời gian</t>
+          <t>Theo dõi tiến độ triển khai, thời gian bắt đầu/kết thúc, số ngày còn lại và trạng thái thực tế của các dự án</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -853,7 +850,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Đã cập nhật bộ lọc &amp; RAG</t>
+          <t>Chuẩn 11 cột thực tế (đã bỏ cột rủi ro RAG)</t>
         </is>
       </c>
     </row>
@@ -883,7 +880,7 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Đã hiển thị cột phân kỳ động, bỏ VNĐ</t>
+          <t>Đã hiển thị cột phân kỳ động, bỏ chữ VNĐ</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1030,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Chuẩn hóa prefix DAN, GT, HD, TT, NT, NV, LDA, LHD</t>
+          <t>Đồng bộ danh mục theo ProductionSeeder</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1045,7 @@
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>1. Mỗi sheet biểu mẫu gồm 3 phần: [1] Bộ lọc &amp; Tiêu chí tra cứu; [2] Biểu mẫu dữ liệu mẫu; [3] Bảng mô tả chi tiết nguồn dữ liệu (Data Mapping từ CSDL / Backend Entity).</t>
+          <t>1. Mỗi sheet biểu mẫu gồm 3 phần: [1] Bộ lọc &amp; Tiêu chí tra cứu; [2] Biểu mẫu dữ liệu mẫu khớp 100% giao diện thực tế phần mềm; [3] Bảng mô tả chi tiết nguồn dữ liệu (Data Mapping từ CSDL / Backend Entity).</t>
         </is>
       </c>
     </row>
@@ -1073,33 +1070,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BÁO CÁO 1 - TIẾN ĐỘ DỰ ÁN</t>
+          <t>Báo cáo 1: Tiến độ Dự án triển khai</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Theo dõi tiến độ tổng thể, mốc thời gian, trạng thái và mức độ cảnh báo rủi ro (RAG) của các dự án</t>
+          <t>Theo dõi tiến độ triển khai thực tế, đơn vị chủ trì, PM phụ trách, thời hạn và trạng thái của các dự án (Khớp 100% UI phần mềm)</t>
         </is>
       </c>
     </row>
@@ -1226,64 +1223,64 @@
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>2. BIỂU MẪU DỮ LIỆU CHI TIẾT (REPORT DATA PREVIEW)</t>
+          <t>2. BIỂU MẪU DỮ LIỆU CHI TIẾT (REPORT DATA PREVIEW - Khớp thực tế UI phần mềm)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>STT</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mã dự án</t>
+          <t>MÃ DỰ ÁN</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Đơn vị chủ trì</t>
+          <t>TÊN DỰ ÁN TRIỂN KHAI</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>PM phụ trách</t>
+          <t>ĐƠN VỊ CHỦ TRÌ</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Loại dự án</t>
+          <t>PM PHỤ TRÁCH</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Ngày bắt đầu</t>
+          <t>LOẠI DỰ ÁN</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Ngày kết thúc</t>
+          <t>NGÀY BẮT ĐẦU</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Tiến độ (%)</t>
+          <t>NGÀY KẾT THÚC</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Thời gian còn lại (ngày)</t>
+          <t>TIẾN ĐỘ</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Trạng thái thực tế</t>
+          <t>THỜI GIAN CÒN LẠI (NGÀY)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Cảnh báo rủi ro (RAG)</t>
+          <t>TRẠNG THÁI THỰC TẾ</t>
         </is>
       </c>
     </row>
@@ -1293,50 +1290,36 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>DAN-2026-001</t>
+          <t>DAN-2026-859</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Trung tâm CNTT</t>
+          <t>Test trạng thái</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Văn A</t>
+          <t>TT CNTT</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Bản quyền phần mềm</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>09/08/2026</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>12/12/2026</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="I14" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="J14" s="9" t="inlineStr">
-        <is>
-          <t>Đang triển khai</t>
-        </is>
-      </c>
-      <c r="K14" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Đúng tiến độ</t>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Ngân hàng số &amp; Thẻ</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
         </is>
       </c>
     </row>
@@ -1346,50 +1329,36 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>DAN-2026-002</t>
+          <t>DAN-2026-595</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Trung tâm CNTT</t>
+          <t>Dự án Hợp nhất (Gộp từ DAN-2026-879 &amp; DAN-2026-503)</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Trần Thị B</t>
+          <t>TT CNTT</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Mua sắm phần cứng</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>01/01/2026</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>85%</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="9" t="inlineStr">
-        <is>
-          <t>Đã hoàn thành</t>
-        </is>
-      </c>
-      <c r="K15" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Hoàn thành</t>
+          <t>Lê Thị Ánh</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Hạ tầng</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr"/>
+      <c r="J15" s="9" t="inlineStr"/>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
         </is>
       </c>
     </row>
@@ -1399,50 +1368,32 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>DAN-2026-003</t>
+          <t>DAN-TEST-NV-593</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Phòng Kế toán</t>
+          <t>Dự án kiểm tra 2 nguồn vốn cùng năm</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Lê Văn C</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Tư vấn</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>15/03/2026</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>15/10/2026</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="I16" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="J16" s="9" t="inlineStr">
-        <is>
-          <t>Đang triển khai</t>
-        </is>
-      </c>
-      <c r="K16" s="22" t="inlineStr">
-        <is>
-          <t>🟡 Nguy cơ chậm</t>
+          <t>TT CNTT</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Hạ tầng</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr"/>
+      <c r="H16" s="9" t="inlineStr"/>
+      <c r="I16" s="9" t="inlineStr"/>
+      <c r="J16" s="9" t="inlineStr"/>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
         </is>
       </c>
     </row>
@@ -1452,251 +1403,269 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>DAN-2026-004</t>
+          <t>DAN-2026-744</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
+          <t>Mua sắm Switch</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>CNTT</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Hạ tầng</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>08/06/2023</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr"/>
+      <c r="I17" s="9" t="inlineStr"/>
+      <c r="J17" s="9" t="inlineStr"/>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>DAN-2026-214</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Nâng cấp Hệ thống QLTT báo cáo Quỹ tín dụng nhân dân (PRMS)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
           <t>Trung tâm CNTT</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Phạm Văn D</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Bảo trì</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>01/02/2026</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>01/08/2026</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="I17" s="9" t="n">
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; Bảo trì</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="J18" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="9" t="inlineStr">
-        <is>
-          <t>Đang triển khai</t>
-        </is>
-      </c>
-      <c r="K17" s="23" t="inlineStr">
-        <is>
-          <t>🔴 Quá hạn</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19"/>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>DAN-2026-232</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Test thông báo Email</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>TT CNTT</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Phạm Huy Nhất</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; Bảo trì</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr"/>
+      <c r="H19" s="9" t="inlineStr"/>
+      <c r="I19" s="9" t="inlineStr"/>
+      <c r="J19" s="9" t="inlineStr"/>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>3. MÔ TẢ CHI TIẾT NGUỒN DỮ LIỆU &amp; LOGIC TÍNH TOÁN (DATA MAPPING)</t>
+      <c r="A20" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>DAN-2026-503</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Test gộp 01</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>TT CNTT</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Xây dựng &amp; Bảo trì</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr"/>
+      <c r="H20" s="9" t="inlineStr"/>
+      <c r="I20" s="9" t="inlineStr"/>
+      <c r="J20" s="9" t="inlineStr"/>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Chuẩn bị đầu tư</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="23" t="n"/>
+      <c r="G21" s="23" t="n"/>
+      <c r="H21" s="23" t="n"/>
+      <c r="I21" s="23" t="n"/>
+      <c r="J21" s="23" t="n"/>
+      <c r="K21" s="23" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>3. MÔ TẢ CHI TIẾT NGUỒN DỮ LIỆU &amp; LOGIC TÍNH TOÁN (DATA MAPPING - Chuẩn 11 cột thực tế)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
-        <is>
-          <t>Tên Cột Hiển Thị</t>
-        </is>
-      </c>
-      <c r="C21" s="25" t="inlineStr">
+      <c r="B25" s="25" t="inlineStr">
+        <is>
+          <t>Tên Cột Hiển Thị Trên UI</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="inlineStr">
         <is>
           <t>Bảng / Entity Nguồn</t>
         </is>
       </c>
-      <c r="D21" s="25" t="inlineStr">
+      <c r="D25" s="25" t="inlineStr">
         <is>
           <t>Trường Dữ Liệu (Field)</t>
         </is>
       </c>
-      <c r="E21" s="25" t="inlineStr">
+      <c r="E25" s="25" t="inlineStr">
         <is>
           <t>Kiểu Dữ Liệu</t>
         </is>
       </c>
-      <c r="F21" s="25" t="inlineStr">
+      <c r="F25" s="25" t="inlineStr">
         <is>
           <t>Logic Lấy Dữ Liệu &amp; Công Thức Tính Toán Chi Tiết</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>Chương trình (System)</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Index tự tăng</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>Số thứ tự dòng trong báo cáo (1, 2, 3...)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Mã dự án</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Bảng DuAns (Entity DuAn)</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>DuAn.Code</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>string (nvarchar)</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Mã định danh duy nhất của dự án. Quy chuẩn định dạng: DAN-[Năm]-[STT 3 số] (ví dụ: DAN-2026-001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Đơn vị chủ trì</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Bảng DuAns (Entity DuAn)</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>DuAn.ToChucThucHien / ChuDauTu</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Đơn vị hoặc phòng ban chủ trì triển khai dự án (mặc định 'Trung tâm CNTT' hoặc lấy từ trường ToChucThucHien)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>PM phụ trách</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Bảng Users (liên kết DuAns.ChuDuAnId)</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>DuAn.ChuDuAn.FullName</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Họ tên người quản lý/phụ trách dự án (User liên kết qua khóa ngoại ChuDuAnId hoặc CreatedByUser)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Loại dự án</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Bảng PhanLoaiDuAns (DanhMuc)</t>
+          <t>Chương trình (System)</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>DuAn.PhanLoaiDuAn.TenPhanLoai</t>
+          <t>Index tự tăng</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Loại dự án: Bảo trì, Mua sắm phần cứng, Bản quyền phần mềm, Tư vấn, Thuê dịch vụ, Khác</t>
+          <t>Số thứ tự dòng trong báo cáo (1, 2, 3...)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Ngày bắt đầu</t>
+          <t>MÃ DỰ ÁN</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -1706,27 +1675,27 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>DuAn.NgayBatDau</t>
+          <t>DuAn.Code</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>DateTime?</t>
+          <t>string (nvarchar)</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Ngày khởi động/bắt đầu dự án theo kế hoạch phê duyệt. Format: dd/MM/yyyy</t>
+          <t>Mã định danh duy nhất của dự án. Quy chuẩn định dạng: DAN-[Năm]-[STT 3 số] (ví dụ: DAN-2026-214)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Ngày kết thúc</t>
+          <t>TÊN DỰ ÁN TRIỂN KHAI</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -1736,97 +1705,97 @@
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>DuAn.NgayKetThuc</t>
+          <t>DuAn.Name</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>DateTime?</t>
+          <t>string (nvarchar)</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Ngày dự kiến hoàn thành dự án theo kế hoạch. Format: dd/MM/yyyy</t>
+          <t>Tên đầy đủ của dự án triển khai</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Tiến độ (%)</t>
+          <t>ĐƠN VỊ CHỦ TRÌ</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Bảng CongViecGoiThaus &amp; DuAns</t>
+          <t>Bảng DuAns (Entity DuAn)</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Tính toán hoặc DuAn.TienDoPhanTram</t>
+          <t>DuAn.ToChucThucHien / ChuDauTu</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Tỷ lệ % hoàn thành dự án. Tính từ tỷ lệ hoàn thành các công việc gói thầu có trọng số, hoặc % giải ngân thực tế</t>
+          <t>Đơn vị hoặc phòng ban chủ trì triển khai dự án (mặc định 'TT CNTT' / 'Trung tâm CNTT' hoặc lấy từ trường ToChucThucHien)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Thời gian còn lại (ngày)</t>
+          <t>PM PHỤ TRÁCH</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Tính toán động</t>
+          <t>Bảng Users (liên kết DuAns.ChuDuAnId)</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>(NgayKetThuc - Today).Days</t>
+          <t>DuAn.ChuDuAn.FullName</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>string</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Số ngày còn lại tính từ ngày hiện tại (Today) đến Ngày kết thúc: Math.Max(0, (NgayKetThuc.Date - DateTime.Today).Days). Nếu đã hoàn thành hoặc quá hạn thì = 0</t>
+          <t>Họ tên người quản lý/phụ trách dự án (User liên kết qua khóa ngoại ChuDuAnId hoặc CreatedByUser.FullName)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Trạng thái thực tế</t>
+          <t>LOẠI DỰ ÁN</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Bảng DuAns (Entity DuAn)</t>
+          <t>Bảng PhanLoaiDuAns (DanhMuc)</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>DuAn.TrangThai / DaKetThuc</t>
+          <t>DuAn.PhanLoaiDuAn.Name</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
@@ -1836,48 +1805,188 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>Trạng thái dự án: 1: Chưa triển khai | 2: Đang triển khai | 3: Tạm dừng | 4: Đã nghiệm thu/hoàn thành | 5: Đã hủy</t>
+          <t>Loại dự án thực tế trong hệ thống: 'Ngân hàng số &amp; Thẻ', 'Hạ tầng', 'Xây dựng &amp; Bảo trì', 'Công nghệ thông tin', 'Hệ thống phần mềm', 'Mạng &amp; An ninh bảo mật'...</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>NGÀY BẮT ĐẦU</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Bảng DuAns (Entity DuAn)</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>DuAn.NgayBatDau</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>DateTime?</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Ngày khởi động/bắt đầu dự án theo kế hoạch. Hiển thị dạng dd/MM/yyyy (để trống nếu chưa nhập)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>NGÀY KẾT THÚC</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Bảng DuAns (Entity DuAn)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>DuAn.NgayKetThuc</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>DateTime?</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Ngày dự kiến hoàn thành dự án theo kế hoạch. Hiển thị dạng dd/MM/yyyy (để trống nếu chưa nhập)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>TIẾN ĐỘ</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Bảng CongViecGoiThaus &amp; DuAns</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Tính toán hoặc DuAn.TienDoPhanTram</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>string/decimal</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Tỷ lệ % hoàn thành dự án (ví dụ: '1%'). Tính từ tỷ lệ hoàn thành các công việc gói thầu có trọng số, hoặc % giải ngân</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>THỜI GIAN CÒN LẠI (NGÀY)</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Tính toán động</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>(NgayKetThuc - Today).Days</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>int?</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Số ngày còn lại tính từ ngày hiện tại (Today) đến Ngày kết thúc: Math.Max(0, (NgayKetThuc.Date - DateTime.Today).Days). Nếu đã đến/quá hạn hiển thị '0'</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>Cảnh báo rủi ro (RAG)</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>Hàm đánh giá rủi ro (Warning Logic)</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>Calculated RAG</t>
-        </is>
-      </c>
-      <c r="E32" s="13" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>TRẠNG THÁI THỰC TẾ</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>Bảng DuAns (Entity DuAn)</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>DuAn.TrangThai / Enum TrangThaiDuAn</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>Quy tắc cảnh báo RAG: 
-- 🟢 Đúng tiến độ: Tiến độ đạt &gt;= kế hoạch hoặc còn hạn &gt; 30 ngày.
-- 🟡 Nguy cơ chậm: Còn &lt; 30 ngày nhưng tiến độ &lt; 70%, hoặc có gói thầu trễ hạn.
-- 🔴 Quá hạn / Rủi ro cao: NgayKetThuc &lt; Today mà TrangThai != 'Đã hoàn thành'.</t>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Trạng thái dự án thực tế: 'Chuẩn bị đầu tư', 'Đang triển khai', 'Nghiệm thu', 'Thanh toán', 'Quyết toán', 'Hoàn thành', 'Tạm dừng', 'Đã gộp'</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>📌 GHI CHÚ ĐIỀU CHỈNH:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>- Đã bổ sung cột [TÊN DỰ ÁN TRIỂN KHAI] ngay sau cột [MÃ DỰ ÁN].</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>- Đã xóa bỏ cột [Cảnh báo rủi ro (RAG)] để đúng 100% với thực trạng giao diện phần mềm đang có.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A20:F20"/>
+  <mergeCells count="4">
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A24:F24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2306,7 +2415,7 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>Tên Cột Hiển Thị</t>
+          <t>Tên Cột Hiển Thị Trên UI</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
@@ -2689,7 +2798,7 @@
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -2947,7 +3056,7 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Đấu thầu rộng rãi qua mạng</t>
+          <t>Đấu thầu rộng rãi</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
@@ -3087,7 +3196,7 @@
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>Chỉ định thầu rút gọn</t>
+          <t>Chỉ định thầu</t>
         </is>
       </c>
       <c r="I16" s="9" t="inlineStr">
@@ -3138,7 +3247,7 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>Tên Cột Hiển Thị</t>
+          <t>Tên Cột Hiển Thị Trên UI</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
@@ -3398,7 +3507,7 @@
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Hình thức lựa chọn nhà thầu: Đấu thầu rộng rãi qua mạng, Chỉ định thầu, Chào hàng cạnh tranh, Mua sắm trực tiếp, Tự thực hiện...</t>
+          <t>Hình thức lựa chọn nhà thầu: Đấu thầu rộng rãi, Chỉ định thầu, Chào hàng cạnh tranh, Mua sắm trực tiếp, Tự thực hiện...</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4139,7 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>Tên Cột Hiển Thị</t>
+          <t>Tên Cột Hiển Thị Trên UI</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
@@ -4711,7 +4820,7 @@
           <t>Đã nhận Thư bảo lãnh tạm ứng</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr">
+      <c r="I14" s="40" t="inlineStr">
         <is>
           <t>🟢 Đã thanh toán</t>
         </is>
@@ -4761,7 +4870,7 @@
           <t>Đã ký Biên bản nghiệm thu bàn giao</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr">
+      <c r="I15" s="41" t="inlineStr">
         <is>
           <t>🟡 Chưa thanh toán</t>
         </is>
@@ -4811,7 +4920,7 @@
           <t>Chờ hết thời hạn bảo hành</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="I16" s="41" t="inlineStr">
         <is>
           <t>🟡 Chưa thanh toán</t>
         </is>
@@ -4839,7 +4948,7 @@
       </c>
       <c r="B20" s="25" t="inlineStr">
         <is>
-          <t>Tên Cột Hiển Thị</t>
+          <t>Tên Cột Hiển Thị Trên UI</t>
         </is>
       </c>
       <c r="C20" s="25" t="inlineStr">
@@ -5204,19 +5313,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="40" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>NGÂN HÀNG HỢP TÁC XÃ VIỆT NAM</t>
         </is>
       </c>
-      <c r="S1" s="41" t="inlineStr">
+      <c r="S1" s="43" t="inlineStr">
         <is>
           <t>Biểu số 02.A</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
         <is>
           <t>TRUNG TÂM CÔNG NGHỆ THÔNG TIN</t>
         </is>
@@ -5224,21 +5333,21 @@
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>TÌNH HÌNH ĐẦU TƯ VÀ HUY ĐỘNG VỐN ĐỂ ĐẦU TƯ VÀO CÁC DỰ ÁN HÌNH THÀNH TSCĐ VÀ XDCB</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="43" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>(Ban hành kèm theo Thông tư số 200/2015/TT-BTC ngày 15/12/2015 của Bộ Tài chính)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="A6" s="46" t="inlineStr">
         <is>
           <t>Kỳ báo cáo: Quý III năm 2026 | Đơn vị tính: Tỷ đồng</t>
         </is>
@@ -5246,231 +5355,231 @@
     </row>
     <row r="7"/>
     <row r="8">
-      <c r="A8" s="45" t="inlineStr">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>TT</t>
         </is>
       </c>
-      <c r="B8" s="45" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Tên dự án</t>
         </is>
       </c>
-      <c r="C8" s="45" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>Quyết định phê duyệt</t>
         </is>
       </c>
-      <c r="D8" s="45" t="inlineStr">
+      <c r="D8" s="47" t="inlineStr">
         <is>
           <t>Tổng mức vốn đầu tư</t>
         </is>
       </c>
-      <c r="E8" s="46" t="n"/>
-      <c r="F8" s="46" t="n"/>
-      <c r="G8" s="46" t="n"/>
-      <c r="H8" s="46" t="n"/>
-      <c r="I8" s="45" t="inlineStr">
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="n"/>
+      <c r="I8" s="47" t="inlineStr">
         <is>
           <t>Thời gian đầu tư theo KH</t>
         </is>
       </c>
-      <c r="J8" s="45" t="inlineStr">
+      <c r="J8" s="47" t="inlineStr">
         <is>
           <t>Nguồn vốn huy động</t>
         </is>
       </c>
-      <c r="K8" s="46" t="n"/>
-      <c r="L8" s="46" t="n"/>
-      <c r="M8" s="45" t="inlineStr">
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="M8" s="47" t="inlineStr">
         <is>
           <t>Giá trị khối lượng thực hiện đến cuối kỳ</t>
         </is>
       </c>
-      <c r="N8" s="46" t="n"/>
-      <c r="O8" s="46" t="n"/>
-      <c r="P8" s="45" t="inlineStr">
+      <c r="N8" s="23" t="n"/>
+      <c r="O8" s="23" t="n"/>
+      <c r="P8" s="47" t="inlineStr">
         <is>
           <t>Giải ngân đến cuối kỳ</t>
         </is>
       </c>
-      <c r="Q8" s="46" t="n"/>
-      <c r="R8" s="46" t="n"/>
-      <c r="S8" s="45" t="inlineStr">
+      <c r="Q8" s="23" t="n"/>
+      <c r="R8" s="23" t="n"/>
+      <c r="S8" s="47" t="inlineStr">
         <is>
           <t>Giá trị tài sản đã hình thành đưa vào sử dụng</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="n"/>
-      <c r="B9" s="46" t="n"/>
-      <c r="C9" s="46" t="n"/>
-      <c r="D9" s="47" t="inlineStr">
+      <c r="A9" s="23" t="n"/>
+      <c r="B9" s="23" t="n"/>
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="48" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="E9" s="47" t="inlineStr">
+      <c r="E9" s="48" t="inlineStr">
         <is>
           <t>Vốn CSH</t>
         </is>
       </c>
-      <c r="F9" s="47" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G9" s="47" t="inlineStr">
+      <c r="G9" s="48" t="inlineStr">
         <is>
           <t>Vốn vay/HĐ</t>
         </is>
       </c>
-      <c r="H9" s="47" t="inlineStr">
+      <c r="H9" s="48" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="I9" s="46" t="n"/>
-      <c r="J9" s="47" t="inlineStr">
+      <c r="I9" s="23" t="n"/>
+      <c r="J9" s="48" t="inlineStr">
         <is>
           <t>Tổng số</t>
         </is>
       </c>
-      <c r="K9" s="47" t="inlineStr">
+      <c r="K9" s="48" t="inlineStr">
         <is>
           <t>Thời hạn vay</t>
         </is>
       </c>
-      <c r="L9" s="47" t="inlineStr">
+      <c r="L9" s="48" t="inlineStr">
         <is>
           <t>Lãi suất (%)</t>
         </is>
       </c>
-      <c r="M9" s="47" t="inlineStr">
+      <c r="M9" s="48" t="inlineStr">
         <is>
           <t>Kỳ trước chuyển sang</t>
         </is>
       </c>
-      <c r="N9" s="47" t="inlineStr">
+      <c r="N9" s="48" t="inlineStr">
         <is>
           <t>Thực hiện trong kỳ</t>
         </is>
       </c>
-      <c r="O9" s="47" t="inlineStr">
+      <c r="O9" s="48" t="inlineStr">
         <is>
           <t>Lũy kế đến cuối kỳ</t>
         </is>
       </c>
-      <c r="P9" s="47" t="inlineStr">
+      <c r="P9" s="48" t="inlineStr">
         <is>
           <t>Kỳ trước chuyển sang</t>
         </is>
       </c>
-      <c r="Q9" s="47" t="inlineStr">
+      <c r="Q9" s="48" t="inlineStr">
         <is>
           <t>Thực hiện trong kỳ</t>
         </is>
       </c>
-      <c r="R9" s="47" t="inlineStr">
+      <c r="R9" s="48" t="inlineStr">
         <is>
           <t>Lũy kế đến cuối kỳ</t>
         </is>
       </c>
-      <c r="S9" s="46" t="n"/>
+      <c r="S9" s="23" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t>(1)</t>
         </is>
       </c>
-      <c r="B10" s="48" t="inlineStr">
+      <c r="B10" s="49" t="inlineStr">
         <is>
           <t>(2)</t>
         </is>
       </c>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>(3)</t>
         </is>
       </c>
-      <c r="D10" s="48" t="inlineStr">
+      <c r="D10" s="49" t="inlineStr">
         <is>
           <t>(4)</t>
         </is>
       </c>
-      <c r="E10" s="48" t="inlineStr">
+      <c r="E10" s="49" t="inlineStr">
         <is>
           <t>(5)</t>
         </is>
       </c>
-      <c r="F10" s="48" t="inlineStr">
+      <c r="F10" s="49" t="inlineStr">
         <is>
           <t>(6)</t>
         </is>
       </c>
-      <c r="G10" s="48" t="inlineStr">
+      <c r="G10" s="49" t="inlineStr">
         <is>
           <t>(7)</t>
         </is>
       </c>
-      <c r="H10" s="48" t="inlineStr">
+      <c r="H10" s="49" t="inlineStr">
         <is>
           <t>(8)</t>
         </is>
       </c>
-      <c r="I10" s="48" t="inlineStr">
+      <c r="I10" s="49" t="inlineStr">
         <is>
           <t>(9)</t>
         </is>
       </c>
-      <c r="J10" s="48" t="inlineStr">
+      <c r="J10" s="49" t="inlineStr">
         <is>
           <t>(10)</t>
         </is>
       </c>
-      <c r="K10" s="48" t="inlineStr">
+      <c r="K10" s="49" t="inlineStr">
         <is>
           <t>(11)</t>
         </is>
       </c>
-      <c r="L10" s="48" t="inlineStr">
+      <c r="L10" s="49" t="inlineStr">
         <is>
           <t>(12)</t>
         </is>
       </c>
-      <c r="M10" s="48" t="inlineStr">
+      <c r="M10" s="49" t="inlineStr">
         <is>
           <t>(13)</t>
         </is>
       </c>
-      <c r="N10" s="48" t="inlineStr">
+      <c r="N10" s="49" t="inlineStr">
         <is>
           <t>(14)</t>
         </is>
       </c>
-      <c r="O10" s="48" t="inlineStr">
+      <c r="O10" s="49" t="inlineStr">
         <is>
           <t>(15)</t>
         </is>
       </c>
-      <c r="P10" s="48" t="inlineStr">
+      <c r="P10" s="49" t="inlineStr">
         <is>
           <t>(16)</t>
         </is>
       </c>
-      <c r="Q10" s="48" t="inlineStr">
+      <c r="Q10" s="49" t="inlineStr">
         <is>
           <t>(17)</t>
         </is>
       </c>
-      <c r="R10" s="48" t="inlineStr">
+      <c r="R10" s="49" t="inlineStr">
         <is>
           <t>(18)</t>
         </is>
       </c>
-      <c r="S10" s="48" t="inlineStr">
+      <c r="S10" s="49" t="inlineStr">
         <is>
           <t>(19)</t>
         </is>
@@ -5920,23 +6029,23 @@
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr"/>
-      <c r="D19" s="49" t="n">
+      <c r="D19" s="50" t="n">
         <v>181.89</v>
       </c>
-      <c r="E19" s="49" t="n">
+      <c r="E19" s="50" t="n">
         <v>181.89</v>
       </c>
-      <c r="F19" s="49" t="n">
+      <c r="F19" s="50" t="n">
         <v>100</v>
       </c>
-      <c r="G19" s="49" t="n">
+      <c r="G19" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="49" t="n">
+      <c r="H19" s="50" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="10" t="inlineStr"/>
-      <c r="J19" s="49" t="n">
+      <c r="J19" s="50" t="n">
         <v>0</v>
       </c>
       <c r="K19" s="11" t="inlineStr">
@@ -5949,25 +6058,25 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M19" s="49" t="n">
+      <c r="M19" s="50" t="n">
         <v>2.32</v>
       </c>
-      <c r="N19" s="49" t="n">
+      <c r="N19" s="50" t="n">
         <v>48.78</v>
       </c>
-      <c r="O19" s="49" t="n">
+      <c r="O19" s="50" t="n">
         <v>51.09</v>
       </c>
-      <c r="P19" s="49" t="n">
+      <c r="P19" s="50" t="n">
         <v>2.32</v>
       </c>
-      <c r="Q19" s="49" t="n">
+      <c r="Q19" s="50" t="n">
         <v>48.78</v>
       </c>
-      <c r="R19" s="49" t="n">
+      <c r="R19" s="50" t="n">
         <v>51.09</v>
       </c>
-      <c r="S19" s="49" t="n">
+      <c r="S19" s="50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6510,23 +6619,23 @@
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr"/>
-      <c r="D29" s="49" t="n">
+      <c r="D29" s="50" t="n">
         <v>72.65000000000001</v>
       </c>
-      <c r="E29" s="49" t="n">
+      <c r="E29" s="50" t="n">
         <v>72.65000000000001</v>
       </c>
-      <c r="F29" s="49" t="n">
+      <c r="F29" s="50" t="n">
         <v>100</v>
       </c>
-      <c r="G29" s="49" t="n">
+      <c r="G29" s="50" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="49" t="n">
+      <c r="H29" s="50" t="n">
         <v>0</v>
       </c>
       <c r="I29" s="10" t="inlineStr"/>
-      <c r="J29" s="49" t="n">
+      <c r="J29" s="50" t="n">
         <v>0</v>
       </c>
       <c r="K29" s="11" t="inlineStr">
@@ -6539,25 +6648,25 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M29" s="49" t="n">
+      <c r="M29" s="50" t="n">
         <v>23.26</v>
       </c>
-      <c r="N29" s="49" t="n">
+      <c r="N29" s="50" t="n">
         <v>21.1</v>
       </c>
-      <c r="O29" s="49" t="n">
+      <c r="O29" s="50" t="n">
         <v>44.34</v>
       </c>
-      <c r="P29" s="49" t="n">
+      <c r="P29" s="50" t="n">
         <v>23.26</v>
       </c>
-      <c r="Q29" s="49" t="n">
+      <c r="Q29" s="50" t="n">
         <v>21.1</v>
       </c>
-      <c r="R29" s="49" t="n">
+      <c r="R29" s="50" t="n">
         <v>44.34</v>
       </c>
-      <c r="S29" s="49" t="n">
+      <c r="S29" s="50" t="n">
         <v>7.64</v>
       </c>
     </row>
@@ -6636,7 +6745,7 @@
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>Tên Cột Hiển Thị</t>
+          <t>Tên Cột Hiển Thị Trên UI</t>
         </is>
       </c>
       <c r="C33" s="25" t="inlineStr">
@@ -7253,7 +7362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -7327,19 +7436,19 @@
           <t>Mã Dự án</t>
         </is>
       </c>
-      <c r="C6" s="50" t="inlineStr">
+      <c r="C6" s="51" t="inlineStr">
         <is>
           <t>DAN-[Năm]-[STT 3 số]</t>
         </is>
       </c>
-      <c r="D6" s="50" t="inlineStr">
-        <is>
-          <t>DAN-2026-001</t>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>DAN-2026-214</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>DAN: Dự án; 2026: Năm tạo; 001: Số thứ tự tự tăng trong năm</t>
+          <t>DAN: Dự án; 2026: Năm tạo; 214: Số thứ tự tự tăng trong năm</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -7387,12 +7496,12 @@
           <t>Số / Mã Hợp đồng</t>
         </is>
       </c>
-      <c r="C8" s="50" t="inlineStr">
+      <c r="C8" s="51" t="inlineStr">
         <is>
           <t>HD-[Năm]-[STT 3 số]</t>
         </is>
       </c>
-      <c r="D8" s="50" t="inlineStr">
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>HD-2026-017</t>
         </is>
@@ -7447,12 +7556,12 @@
           <t>Mã Nhà thầu / Đối tác</t>
         </is>
       </c>
-      <c r="C10" s="50" t="inlineStr">
+      <c r="C10" s="51" t="inlineStr">
         <is>
           <t>NT-[Tên viết tắt]</t>
         </is>
       </c>
-      <c r="D10" s="50" t="inlineStr">
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>NT-CMC, NT-FPT</t>
         </is>
@@ -7507,19 +7616,19 @@
           <t>Mã Loại Dự án</t>
         </is>
       </c>
-      <c r="C12" s="50" t="inlineStr">
+      <c r="C12" s="51" t="inlineStr">
         <is>
           <t>LDA-[Tên viết tắt]</t>
         </is>
       </c>
-      <c r="D12" s="50" t="inlineStr">
-        <is>
-          <t>LDA-BT, LDA-MSPC, LDA-BQPM</t>
+      <c r="D12" s="51" t="inlineStr">
+        <is>
+          <t>LDA-NHST, LDA-HT, LDA-XDCB</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>LDA: Loại dự án; BT: Bảo trì, MSPC: Mua sắm phần cứng, BQPM: Bản quyền PM</t>
+          <t>LDA: Loại dự án; NHST: Ngân hàng số &amp; Thẻ, HT: Hạ tầng, XDCB: Xây dựng &amp; Bảo trì</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
@@ -7563,7 +7672,7 @@
     <row r="16">
       <c r="A16" s="28" t="inlineStr">
         <is>
-          <t>2. DANH MỤC LOẠI DỰ ÁN &amp; MÃ VIẾT TẮT</t>
+          <t>2. DANH MỤC LOẠI DỰ ÁN &amp; MÃ VIẾT TẮT (Chuẩn CSDL Production)</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7689,7 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Tên Loại Dự Án</t>
+          <t>Tên Loại Dự Án (Hiển thị UI)</t>
         </is>
       </c>
       <c r="D17" s="27" t="inlineStr">
@@ -7593,19 +7702,19 @@
       <c r="A18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="50" t="inlineStr">
-        <is>
-          <t>LDA-BT</t>
+      <c r="B18" s="51" t="inlineStr">
+        <is>
+          <t>PL_DIGITAL_BANKING</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Bảo trì</t>
+          <t>Ngân hàng số &amp; Thẻ</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Bảo trì, bảo dưỡng hệ thống công nghệ thông tin, phần cứng và hạ tầng</t>
+          <t>Dự án liên quan đến sản phẩm, kênh số, Core banking và dịch vụ thẻ</t>
         </is>
       </c>
     </row>
@@ -7615,17 +7724,17 @@
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>LDA-MSPC</t>
+          <t>PL_HA_TANG</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Mua sắm phần cứng</t>
+          <t>Hạ tầng</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Mua sắm máy chủ, thiết bị mạng, máy trạm, thiết bị lưu trữ và phụ kiện</t>
+          <t>Dự án đầu tư máy chủ, đường truyền, tủ rack, hệ thống mạng và trung tâm dữ liệu</t>
         </is>
       </c>
     </row>
@@ -7633,19 +7742,19 @@
       <c r="A20" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="50" t="inlineStr">
-        <is>
-          <t>LDA-BQPM</t>
+      <c r="B20" s="51" t="inlineStr">
+        <is>
+          <t>PL_XDCB</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Bản quyền phần mềm</t>
+          <t>Xây dựng &amp; Bảo trì</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Mua sắm, gia hạn giấy phép bản quyền phần mềm (License / SLA)</t>
+          <t>Dự án xây dựng cơ bản, nâng cấp bảo trì hạ tầng vật lý và phòng máy</t>
         </is>
       </c>
     </row>
@@ -7655,17 +7764,17 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>LDA-TV</t>
+          <t>PL_CNTT</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Tư vấn</t>
+          <t>Công nghệ thông tin</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Tư vấn lập báo cáo khả thi, tư vấn thiết kế thi công, tư vấn giám sát CNTT</t>
+          <t>Dự án công nghệ thông tin tổng thể</t>
         </is>
       </c>
     </row>
@@ -7673,19 +7782,19 @@
       <c r="A22" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B22" s="50" t="inlineStr">
-        <is>
-          <t>LDA-TDV</t>
+      <c r="B22" s="51" t="inlineStr">
+        <is>
+          <t>PL_HTPM</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Thuê dịch vụ</t>
+          <t>Hệ thống phần mềm</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Thuê dịch vụ đường truyền, Cloud, dịch vụ trung tâm dữ liệu, bảo mật SOC</t>
+          <t>Dự án mua sắm, phát triển hoặc nâng cấp các hệ thống ứng dụng phần mềm</t>
         </is>
       </c>
     </row>
@@ -7695,126 +7804,166 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>LDA-KHAC</t>
+          <t>PL_SECURITY</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
+          <t>Mạng &amp; An ninh bảo mật</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Dự án trang bị tường lửa, giải pháp SIEM, SOC, kiểm thử xâm nhập ATTT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>PL_MSHH_DV</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Mua sắm hàng hóa &amp; Dịch vụ</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Mua sắm hàng hóa vật tư và thuê dịch vụ chuyên gia CNTT</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>PL_KHAC</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
           <t>Khác</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Các dự án đặc thù khác ngoài các danh mục trên</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Các dự án đặc thù khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>3. BẢNG TRA CỨU TRẠNG THÁI THỰC HIỆN CÁC ĐỐI TƯỢNG</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="25" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B27" s="25" t="inlineStr">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>Đối Tượng</t>
         </is>
       </c>
-      <c r="C27" s="25" t="inlineStr">
+      <c r="C29" s="25" t="inlineStr">
         <is>
           <t>Giá Trị Trạng Thái Trong DB (Enum / Id)</t>
         </is>
       </c>
-      <c r="D27" s="25" t="inlineStr">
-        <is>
-          <t>Tên Hiển Thị Chuẩn Trên Báo Cáo</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Dự án (DuAn)</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>1: Chưa triển khai | 2: Đang triển khai | 3: Tạm dừng | 4: Hoàn thành | 5: Đã hủy</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>Chưa triển khai | Đang triển khai | Tạm dừng | Đã nghiệm thu/hoàn thành | Đã hủy</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Gói thầu (GoiThau)</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>1: Chưa LCNT | 2: Đang LCNT | 3: Đã phê duyệt KQLCNT | 4: Đã ký HĐ | 5: Hoàn thành | 6: Đã hủy</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Chưa LCNT | Đang tổ chức LCNT | Đã phê duyệt KQLCNT | Đã hoàn thành LCNT | Đã hủy</t>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>Tên Hiển Thị Chuẩn Trên Báo Cáo &amp; UI</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Hợp đồng (HopDong)</t>
+          <t>Dự án (DuAn)</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>IsActive = true/false, ExpiredDate so với Today, DaKetThuc</t>
+          <t>1: Chuẩn bị đầu tư (Draft/Submitted) | 4: Đang triển khai | 5: Nghiệm thu | 6: Thanh toán | 7: Quyết toán | 8: Hoàn thành | 9: Tạm dừng | 10: Đã gộp</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>Đang thực hiện | Sắp hết hạn | Đã hết hạn | Đã thanh lý/hoàn thành</t>
+          <t>Chuẩn bị đầu tư | Đang triển khai | Nghiệm thu | Thanh toán | Quyết toán | Hoàn thành | Tạm dừng | Đã gộp</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Gói thầu (GoiThau)</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>1: Chưa LCNT | 2: Đang LCNT | 3: Đã phê duyệt KQLCNT | 4: Đã ký HĐ | 5: Hoàn thành | 6: Đã hủy</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Chưa LCNT | Đang tổ chức LCNT | Đã phê duyệt KQLCNT | Đã hoàn thành LCNT | Đã hủy</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Hợp đồng (HopDong)</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>IsActive = true/false, ExpiredDate so với Today, DaKetThuc</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Đang thực hiện | Sắp hết hạn | Đã hết hạn | Đã thanh lý/hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Đợt thanh toán (DotThanhToan)</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>IsPaid = false (Chưa thanh toán) | IsPaid = true (Đã thanh toán)</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>🟡 Chưa thanh toán | 🟢 Đã thanh toán</t>
         </is>
@@ -7823,7 +7972,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>